<commit_message>
Emis Exam Server 8.0 Upgraded
</commit_message>
<xml_diff>
--- a/RESULTS/2026/CLASS/JSS1/FIRST/English_language/results.xlsx
+++ b/RESULTS/2026/CLASS/JSS1/FIRST/English_language/results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,72 +490,6 @@
       <c r="O1" t="inlineStr">
         <is>
           <t>Termination Reason</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Abbas Bello Aisha</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>std015</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>JSS1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>JSS1A</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>ENGLISH LANGUAGE</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>FIRST</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>18</v>
-      </c>
-      <c r="I2" t="n">
-        <v>60</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>65</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-09-14 15:36</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
         </is>
       </c>
     </row>

</xml_diff>